<commit_message>
added benchmark_runner & plans for future scripts, amended AR1 script
</commit_message>
<xml_diff>
--- a/data/ar-process/cv_results.xlsx
+++ b/data/ar-process/cv_results.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly_naive" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly_cmp" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly_naive" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly_cmp" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_5day" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_5day_naive" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_5day_cmp" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_7day" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_7day_naive" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_7day_cmp" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly_naive" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly_cmp" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Monthly" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Monthly_naive" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Monthly_cmp" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Weekly" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Weekly_naive" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Weekly_cmp" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Daily_5day" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Daily_5day_naive" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Daily_5day_cmp" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Daily_7day" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Daily_7day_naive" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Daily_7day_cmp" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Quarterly" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Quarterly_naive" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Quarterly_cmp" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,16 +31,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -51,7 +48,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -59,21 +56,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,36 +427,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE</t>
         </is>
@@ -682,16 +670,16 @@
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>634.6682855273244</v>
+        <v>634.6682855273415</v>
       </c>
       <c r="D11" t="n">
-        <v>634.6682855273244</v>
+        <v>634.6682855273415</v>
       </c>
       <c r="E11" t="n">
-        <v>8.044403655527697</v>
+        <v>8.044403655527892</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1158081270443778</v>
+        <v>0.1158081270443809</v>
       </c>
     </row>
     <row r="12">
@@ -704,16 +692,16 @@
         <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>1066.498162490569</v>
+        <v>1066.498162490575</v>
       </c>
       <c r="D12" t="n">
-        <v>931.9092483923808</v>
+        <v>931.9092483923876</v>
       </c>
       <c r="E12" t="n">
-        <v>11.24945328796923</v>
+        <v>11.2494532879693</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1946042641656243</v>
+        <v>0.1946042641656254</v>
       </c>
     </row>
     <row r="13">
@@ -726,16 +714,16 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>1266.715740594028</v>
+        <v>1266.715740594034</v>
       </c>
       <c r="D13" t="n">
-        <v>1127.043865693625</v>
+        <v>1127.043865693632</v>
       </c>
       <c r="E13" t="n">
-        <v>12.24268904585004</v>
+        <v>12.2426890458501</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2311380303081343</v>
+        <v>0.2311380303081354</v>
       </c>
     </row>
     <row r="14">
@@ -823,7 +811,7 @@
         <v>1.917018841290859</v>
       </c>
       <c r="F17" t="n">
-        <v>0.04025625817740449</v>
+        <v>0.04025715601658439</v>
       </c>
     </row>
     <row r="18">
@@ -836,16 +824,16 @@
         <v>6</v>
       </c>
       <c r="C18" t="n">
-        <v>3.70288527176887</v>
+        <v>3.702885271768876</v>
       </c>
       <c r="D18" t="n">
-        <v>3.424022930338694</v>
+        <v>3.4240229303387</v>
       </c>
       <c r="E18" t="n">
-        <v>3.671861741675678</v>
+        <v>3.671861741675683</v>
       </c>
       <c r="F18" t="n">
-        <v>0.07912604394682909</v>
+        <v>0.07912780870256217</v>
       </c>
     </row>
     <row r="19">
@@ -858,16 +846,82 @@
         <v>12</v>
       </c>
       <c r="C19" t="n">
-        <v>3.495400502048368</v>
+        <v>3.495400502048374</v>
       </c>
       <c r="D19" t="n">
-        <v>3.131166137714825</v>
+        <v>3.131166137714831</v>
       </c>
       <c r="E19" t="n">
-        <v>3.267081114533197</v>
+        <v>3.267081114533203</v>
       </c>
       <c r="F19" t="n">
-        <v>0.07469235297282828</v>
+        <v>0.07469401884352714</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>UNRATE</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.2545912035899315</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.2545912035899315</v>
+      </c>
+      <c r="E20" t="n">
+        <v>5.947711707369864</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.04495128187148163</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>UNRATE</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1.735201261791611</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.545951659656554</v>
+      </c>
+      <c r="E21" t="n">
+        <v>16.2594830752253</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.3063716260526371</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>UNRATE</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>12</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.590744317708521</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.366846377721946</v>
+      </c>
+      <c r="E22" t="n">
+        <v>19.61017914068867</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.2808659341033154</v>
       </c>
     </row>
   </sheetData>
@@ -885,32 +939,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE</t>
         </is>
@@ -926,16 +980,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.006082266611817389</v>
+        <v>0.006082266646984458</v>
       </c>
       <c r="D2" t="n">
-        <v>0.006082266611817389</v>
+        <v>0.006082266646984458</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1420417336309575</v>
+        <v>0.1420417344588761</v>
       </c>
       <c r="F2" t="n">
-        <v>0.001321436497114544</v>
+        <v>0.001321436504754961</v>
       </c>
     </row>
     <row r="3">
@@ -948,16 +1002,16 @@
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>0.06113696424388856</v>
+        <v>0.06113696409785259</v>
       </c>
       <c r="D3" t="n">
-        <v>0.05242994101516534</v>
+        <v>0.05242994109076397</v>
       </c>
       <c r="E3" t="n">
-        <v>1.231395130481135</v>
+        <v>1.231395132200785</v>
       </c>
       <c r="F3" t="n">
-        <v>0.01328264955003699</v>
+        <v>0.01328264951830914</v>
       </c>
     </row>
     <row r="4">
@@ -970,16 +1024,16 @@
         <v>30</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1023881400825412</v>
+        <v>0.1023881390600113</v>
       </c>
       <c r="D4" t="n">
-        <v>0.08979129334577814</v>
+        <v>0.08979129248471759</v>
       </c>
       <c r="E4" t="n">
-        <v>2.115500600389232</v>
+        <v>2.115500579631561</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02224490207546474</v>
+        <v>0.02224490185330935</v>
       </c>
     </row>
   </sheetData>
@@ -997,32 +1051,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE</t>
         </is>
@@ -1109,57 +1163,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE_ar1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE_ar1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE_ar1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE_ar1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>mean_RMSE_naive</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>mean_MAE_naive</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mean_MAPE_naive</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>NRMSE_naive</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>rmse_improvement_pct</t>
         </is>
@@ -1175,16 +1229,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.006082266611817389</v>
+        <v>0.006082266646984458</v>
       </c>
       <c r="D2" t="n">
-        <v>0.006082266611817389</v>
+        <v>0.006082266646984458</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1420417336309575</v>
+        <v>0.1420417344588761</v>
       </c>
       <c r="F2" t="n">
-        <v>0.001321436497114544</v>
+        <v>0.001321436504754961</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -1210,16 +1264,16 @@
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>0.06113696424388856</v>
+        <v>0.06113696409785259</v>
       </c>
       <c r="D3" t="n">
-        <v>0.05242994101516534</v>
+        <v>0.05242994109076397</v>
       </c>
       <c r="E3" t="n">
-        <v>1.231395130481135</v>
+        <v>1.231395132200785</v>
       </c>
       <c r="F3" t="n">
-        <v>0.01328264955003699</v>
+        <v>0.01328264951830914</v>
       </c>
       <c r="G3" t="n">
         <v>0.02078724071164026</v>
@@ -1234,7 +1288,7 @@
         <v>0.004516247034830158</v>
       </c>
       <c r="K3" t="n">
-        <v>-194.1081266724044</v>
+        <v>-194.1081259698775</v>
       </c>
     </row>
     <row r="4">
@@ -1247,16 +1301,16 @@
         <v>30</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1023881400825412</v>
+        <v>0.1023881390600113</v>
       </c>
       <c r="D4" t="n">
-        <v>0.08979129334577814</v>
+        <v>0.08979129248471759</v>
       </c>
       <c r="E4" t="n">
-        <v>2.115500600389232</v>
+        <v>2.115500579631561</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02224490207546474</v>
+        <v>0.02224490185330935</v>
       </c>
       <c r="G4" t="n">
         <v>0.0552332525282896</v>
@@ -1271,7 +1325,7 @@
         <v>0.01200000598517292</v>
       </c>
       <c r="K4" t="n">
-        <v>-85.37409150420687</v>
+        <v>-85.37408965291289</v>
       </c>
     </row>
   </sheetData>
@@ -1289,32 +1343,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE</t>
         </is>
@@ -1374,16 +1428,16 @@
         <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>763.7905735096841</v>
+        <v>763.7905735096838</v>
       </c>
       <c r="D4" t="n">
-        <v>634.4764346421958</v>
+        <v>634.4764346421956</v>
       </c>
       <c r="E4" t="n">
         <v>2.730431956591123</v>
       </c>
       <c r="F4" t="n">
-        <v>0.09854610934403049</v>
+        <v>0.09854610934403045</v>
       </c>
     </row>
   </sheetData>
@@ -1401,32 +1455,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE</t>
         </is>
@@ -1513,57 +1567,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE_ar1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE_ar1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE_ar1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE_ar1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>mean_RMSE_naive</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>mean_MAE_naive</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mean_MAPE_naive</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>NRMSE_naive</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>rmse_improvement_pct</t>
         </is>
@@ -1653,16 +1707,16 @@
         <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>763.7905735096841</v>
+        <v>763.7905735096838</v>
       </c>
       <c r="D4" t="n">
-        <v>634.4764346421958</v>
+        <v>634.4764346421956</v>
       </c>
       <c r="E4" t="n">
         <v>2.730431956591123</v>
       </c>
       <c r="F4" t="n">
-        <v>0.09854610934403049</v>
+        <v>0.09854610934403045</v>
       </c>
       <c r="G4" t="n">
         <v>1203.375802487449</v>
@@ -1677,7 +1731,7 @@
         <v>0.155262460060179</v>
       </c>
       <c r="K4" t="n">
-        <v>36.52933921964495</v>
+        <v>36.52933921964497</v>
       </c>
     </row>
   </sheetData>
@@ -1691,36 +1745,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE</t>
         </is>
@@ -2075,7 +2129,7 @@
         <v>1.575255537353999</v>
       </c>
       <c r="F17" t="n">
-        <v>0.03307113822496906</v>
+        <v>0.03307187581373083</v>
       </c>
     </row>
     <row r="18">
@@ -2097,7 +2151,7 @@
         <v>3.171083635776957</v>
       </c>
       <c r="F18" t="n">
-        <v>0.06859819727529401</v>
+        <v>0.06859972722745482</v>
       </c>
     </row>
     <row r="19">
@@ -2119,7 +2173,73 @@
         <v>2.693134053725931</v>
       </c>
       <c r="F19" t="n">
-        <v>0.06217462269293468</v>
+        <v>0.06217600937949664</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>UNRATE</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.2600000000000001</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.2600000000000001</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6.071287595877761</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.04590627296538471</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>UNRATE</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1.751931709556651</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="E21" t="n">
+        <v>16.59154650875184</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.3093255972139257</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>UNRATE</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>12</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.612658303096963</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.386666666666667</v>
+      </c>
+      <c r="E22" t="n">
+        <v>20.13001357404949</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.2847351240840896</v>
       </c>
     </row>
   </sheetData>
@@ -2133,61 +2253,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE_ar1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE_ar1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE_ar1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE_ar1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>mean_RMSE_naive</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>mean_MAE_naive</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mean_MAPE_naive</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>NRMSE_naive</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>rmse_improvement_pct</t>
         </is>
@@ -2536,16 +2656,16 @@
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>634.6682855273244</v>
+        <v>634.6682855273415</v>
       </c>
       <c r="D11" t="n">
-        <v>634.6682855273244</v>
+        <v>634.6682855273415</v>
       </c>
       <c r="E11" t="n">
-        <v>8.044403655527697</v>
+        <v>8.044403655527892</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1158081270443778</v>
+        <v>0.1158081270443809</v>
       </c>
       <c r="G11" t="n">
         <v>560</v>
@@ -2560,7 +2680,7 @@
         <v>0.1021833808679565</v>
       </c>
       <c r="K11" t="n">
-        <v>-13.33362241559365</v>
+        <v>-13.33362241559669</v>
       </c>
     </row>
     <row r="12">
@@ -2573,16 +2693,16 @@
         <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>1066.498162490569</v>
+        <v>1066.498162490575</v>
       </c>
       <c r="D12" t="n">
-        <v>931.9092483923808</v>
+        <v>931.9092483923876</v>
       </c>
       <c r="E12" t="n">
-        <v>11.24945328796923</v>
+        <v>11.2494532879693</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1946042641656243</v>
+        <v>0.1946042641656254</v>
       </c>
       <c r="G12" t="n">
         <v>1032.451763600303</v>
@@ -2597,7 +2717,7 @@
         <v>0.1883918067638628</v>
       </c>
       <c r="K12" t="n">
-        <v>-3.297626106186483</v>
+        <v>-3.297626106187078</v>
       </c>
     </row>
     <row r="13">
@@ -2610,16 +2730,16 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>1266.715740594028</v>
+        <v>1266.715740594034</v>
       </c>
       <c r="D13" t="n">
-        <v>1127.043865693625</v>
+        <v>1127.043865693632</v>
       </c>
       <c r="E13" t="n">
-        <v>12.24268904585004</v>
+        <v>12.2426890458501</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2311380303081343</v>
+        <v>0.2311380303081354</v>
       </c>
       <c r="G13" t="n">
         <v>1223.888122344222</v>
@@ -2634,7 +2754,7 @@
         <v>0.2233232609736925</v>
       </c>
       <c r="K13" t="n">
-        <v>-3.499308267472589</v>
+        <v>-3.499308267473091</v>
       </c>
     </row>
     <row r="14">
@@ -2767,7 +2887,7 @@
         <v>1.917018841290859</v>
       </c>
       <c r="F17" t="n">
-        <v>0.04025625817740449</v>
+        <v>0.04025715601658439</v>
       </c>
       <c r="G17" t="n">
         <v>1.547639999999998</v>
@@ -2779,7 +2899,7 @@
         <v>1.575255537353999</v>
       </c>
       <c r="J17" t="n">
-        <v>0.03307113822496906</v>
+        <v>0.03307187581373083</v>
       </c>
       <c r="K17" t="n">
         <v>-21.72625539392708</v>
@@ -2795,16 +2915,16 @@
         <v>6</v>
       </c>
       <c r="C18" t="n">
-        <v>3.70288527176887</v>
+        <v>3.702885271768876</v>
       </c>
       <c r="D18" t="n">
-        <v>3.424022930338694</v>
+        <v>3.4240229303387</v>
       </c>
       <c r="E18" t="n">
-        <v>3.671861741675678</v>
+        <v>3.671861741675683</v>
       </c>
       <c r="F18" t="n">
-        <v>0.07912604394682909</v>
+        <v>0.07912780870256217</v>
       </c>
       <c r="G18" t="n">
         <v>3.210210465359186</v>
@@ -2816,10 +2936,10 @@
         <v>3.171083635776957</v>
       </c>
       <c r="J18" t="n">
-        <v>0.06859819727529401</v>
+        <v>0.06859972722745482</v>
       </c>
       <c r="K18" t="n">
-        <v>-15.34711856826992</v>
+        <v>-15.3471185682701</v>
       </c>
     </row>
     <row r="19">
@@ -2832,16 +2952,16 @@
         <v>12</v>
       </c>
       <c r="C19" t="n">
-        <v>3.495400502048368</v>
+        <v>3.495400502048374</v>
       </c>
       <c r="D19" t="n">
-        <v>3.131166137714825</v>
+        <v>3.131166137714831</v>
       </c>
       <c r="E19" t="n">
-        <v>3.267081114533197</v>
+        <v>3.267081114533203</v>
       </c>
       <c r="F19" t="n">
-        <v>0.07469235297282828</v>
+        <v>0.07469401884352714</v>
       </c>
       <c r="G19" t="n">
         <v>2.909604514060638</v>
@@ -2853,10 +2973,121 @@
         <v>2.693134053725931</v>
       </c>
       <c r="J19" t="n">
-        <v>0.06217462269293468</v>
+        <v>0.06217600937949664</v>
       </c>
       <c r="K19" t="n">
-        <v>-20.13318253930648</v>
+        <v>-20.13318253930667</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>UNRATE</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.2545912035899315</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.2545912035899315</v>
+      </c>
+      <c r="E20" t="n">
+        <v>5.947711707369864</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.04495128187148163</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.2600000000000001</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.2600000000000001</v>
+      </c>
+      <c r="I20" t="n">
+        <v>6.071287595877761</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.04590627296538471</v>
+      </c>
+      <c r="K20" t="n">
+        <v>2.08030631156486</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>UNRATE</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1.735201261791611</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.545951659656554</v>
+      </c>
+      <c r="E21" t="n">
+        <v>16.2594830752253</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.3063716260526371</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1.751931709556651</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="I21" t="n">
+        <v>16.59154650875184</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.3093255972139257</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.9549714565800138</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>UNRATE</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>12</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.590744317708521</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.366846377721946</v>
+      </c>
+      <c r="E22" t="n">
+        <v>19.61017914068867</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.2808659341033154</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1.612658303096963</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1.386666666666667</v>
+      </c>
+      <c r="I22" t="n">
+        <v>20.13001357404949</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.2847351240840896</v>
+      </c>
+      <c r="K22" t="n">
+        <v>1.358873441841874</v>
       </c>
     </row>
   </sheetData>
@@ -2874,32 +3105,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE</t>
         </is>
@@ -2986,32 +3217,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE</t>
         </is>
@@ -3098,57 +3329,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE_ar1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE_ar1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE_ar1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE_ar1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>mean_RMSE_naive</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>mean_MAE_naive</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mean_MAPE_naive</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>NRMSE_naive</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>rmse_improvement_pct</t>
         </is>
@@ -3280,32 +3511,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE</t>
         </is>
@@ -3453,16 +3684,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7924269433681062</v>
+        <v>0.792426943404088</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7924269433681062</v>
+        <v>0.792426943404088</v>
       </c>
       <c r="E8" t="n">
-        <v>0.538167722454408</v>
+        <v>0.5381677224789044</v>
       </c>
       <c r="F8" t="n">
-        <v>0.00507239804843733</v>
+        <v>0.005072398048667654</v>
       </c>
     </row>
     <row r="9">
@@ -3475,16 +3706,16 @@
         <v>10</v>
       </c>
       <c r="C9" t="n">
-        <v>1.097624307984183</v>
+        <v>1.097624307853077</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9050791234640021</v>
+        <v>0.9050791233244733</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6135875745117074</v>
+        <v>0.613587574416663</v>
       </c>
       <c r="F9" t="n">
-        <v>0.007025994565596231</v>
+        <v>0.007025994564757009</v>
       </c>
     </row>
     <row r="10">
@@ -3497,16 +3728,16 @@
         <v>20</v>
       </c>
       <c r="C10" t="n">
-        <v>1.554315871660555</v>
+        <v>1.554315871593327</v>
       </c>
       <c r="D10" t="n">
-        <v>1.231759421181502</v>
+        <v>1.231759421152263</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8250890087930008</v>
+        <v>0.8250890087744809</v>
       </c>
       <c r="F10" t="n">
-        <v>0.009949319442062133</v>
+        <v>0.0099493194416318</v>
       </c>
     </row>
     <row r="11">
@@ -3585,16 +3816,16 @@
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>0.01747315987143401</v>
+        <v>0.01747315988318887</v>
       </c>
       <c r="D14" t="n">
-        <v>0.01747315987143401</v>
+        <v>0.01747315988318887</v>
       </c>
       <c r="E14" t="n">
-        <v>3.341705760692875</v>
+        <v>3.341705762840536</v>
       </c>
       <c r="F14" t="n">
-        <v>0.02056297362692558</v>
+        <v>0.02056297364075907</v>
       </c>
     </row>
     <row r="15">
@@ -3607,16 +3838,16 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>0.05034918425121487</v>
+        <v>0.05034918424513433</v>
       </c>
       <c r="D15" t="n">
-        <v>0.04308692974909108</v>
+        <v>0.04308692974908783</v>
       </c>
       <c r="E15" t="n">
-        <v>8.030830837844054</v>
+        <v>8.030830838536557</v>
       </c>
       <c r="F15" t="n">
-        <v>0.05925253105407426</v>
+        <v>0.05925253104691848</v>
       </c>
     </row>
     <row r="16">
@@ -3629,16 +3860,16 @@
         <v>20</v>
       </c>
       <c r="C16" t="n">
-        <v>0.04858692400488318</v>
+        <v>0.04858692404786112</v>
       </c>
       <c r="D16" t="n">
-        <v>0.04164247100686599</v>
+        <v>0.04164247103769998</v>
       </c>
       <c r="E16" t="n">
-        <v>7.732248593931897</v>
+        <v>7.73224860067946</v>
       </c>
       <c r="F16" t="n">
-        <v>0.05717864680899615</v>
+        <v>0.05717864685957397</v>
       </c>
     </row>
   </sheetData>
@@ -3656,32 +3887,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE</t>
         </is>
@@ -4032,57 +4263,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>horizon</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_RMSE_ar1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_MAE_ar1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean_MAPE_ar1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>NRMSE_ar1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>mean_RMSE_naive</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>mean_MAE_naive</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mean_MAPE_naive</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>NRMSE_naive</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>rmse_improvement_pct</t>
         </is>
@@ -4320,16 +4551,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7924269433681062</v>
+        <v>0.792426943404088</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7924269433681062</v>
+        <v>0.792426943404088</v>
       </c>
       <c r="E8" t="n">
-        <v>0.538167722454408</v>
+        <v>0.5381677224789044</v>
       </c>
       <c r="F8" t="n">
-        <v>0.00507239804843733</v>
+        <v>0.005072398048667654</v>
       </c>
       <c r="G8" t="n">
         <v>0.7924999999999969</v>
@@ -4344,7 +4575,7 @@
         <v>0.005072865690685148</v>
       </c>
       <c r="K8" t="n">
-        <v>0.009218502446778864</v>
+        <v>0.009218497906478025</v>
       </c>
     </row>
     <row r="9">
@@ -4357,16 +4588,16 @@
         <v>10</v>
       </c>
       <c r="C9" t="n">
-        <v>1.097624307984183</v>
+        <v>1.097624307853077</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9050791234640021</v>
+        <v>0.9050791233244733</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6135875745117074</v>
+        <v>0.613587574416663</v>
       </c>
       <c r="F9" t="n">
-        <v>0.007025994565596231</v>
+        <v>0.007025994564757009</v>
       </c>
       <c r="G9" t="n">
         <v>1.0936919668052</v>
@@ -4381,7 +4612,7 @@
         <v>0.007000823286541425</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.3595474135620085</v>
+        <v>-0.3595474015745368</v>
       </c>
     </row>
     <row r="10">
@@ -4394,16 +4625,16 @@
         <v>20</v>
       </c>
       <c r="C10" t="n">
-        <v>1.554315871660555</v>
+        <v>1.554315871593327</v>
       </c>
       <c r="D10" t="n">
-        <v>1.231759421181502</v>
+        <v>1.231759421152263</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8250890087930008</v>
+        <v>0.8250890087744809</v>
       </c>
       <c r="F10" t="n">
-        <v>0.009949319442062133</v>
+        <v>0.0099493194416318</v>
       </c>
       <c r="G10" t="n">
         <v>1.432969772221878</v>
@@ -4418,7 +4649,7 @@
         <v>0.00917257185273603</v>
       </c>
       <c r="K10" t="n">
-        <v>-8.468154862089323</v>
+        <v>-8.468154857397808</v>
       </c>
     </row>
     <row r="11">
@@ -4542,16 +4773,16 @@
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>0.01747315987143401</v>
+        <v>0.01747315988318887</v>
       </c>
       <c r="D14" t="n">
-        <v>0.01747315987143401</v>
+        <v>0.01747315988318887</v>
       </c>
       <c r="E14" t="n">
-        <v>3.341705760692875</v>
+        <v>3.341705762840536</v>
       </c>
       <c r="F14" t="n">
-        <v>0.02056297362692558</v>
+        <v>0.02056297364075907</v>
       </c>
       <c r="G14" t="n">
         <v>0.01750000000000002</v>
@@ -4566,7 +4797,7 @@
         <v>0.02059455994902799</v>
       </c>
       <c r="K14" t="n">
-        <v>0.1533721632343156</v>
+        <v>0.1533720960636815</v>
       </c>
     </row>
     <row r="15">
@@ -4579,16 +4810,16 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>0.05034918425121487</v>
+        <v>0.05034918424513433</v>
       </c>
       <c r="D15" t="n">
-        <v>0.04308692974909108</v>
+        <v>0.04308692974908783</v>
       </c>
       <c r="E15" t="n">
-        <v>8.030830837844054</v>
+        <v>8.030830838536557</v>
       </c>
       <c r="F15" t="n">
-        <v>0.05925253105407426</v>
+        <v>0.05925253104691848</v>
       </c>
       <c r="G15" t="n">
         <v>0.04968532572900335</v>
@@ -4603,7 +4834,7 @@
         <v>0.05847128110359664</v>
       </c>
       <c r="K15" t="n">
-        <v>-1.336125933504761</v>
+        <v>-1.336125921266649</v>
       </c>
     </row>
     <row r="16">
@@ -4616,16 +4847,16 @@
         <v>20</v>
       </c>
       <c r="C16" t="n">
-        <v>0.04858692400488318</v>
+        <v>0.04858692404786112</v>
       </c>
       <c r="D16" t="n">
-        <v>0.04164247100686599</v>
+        <v>0.04164247103769998</v>
       </c>
       <c r="E16" t="n">
-        <v>7.732248593931897</v>
+        <v>7.73224860067946</v>
       </c>
       <c r="F16" t="n">
-        <v>0.05717864680899615</v>
+        <v>0.05717864685957397</v>
       </c>
       <c r="G16" t="n">
         <v>0.04787544165063147</v>
@@ -4640,7 +4871,7 @@
         <v>0.05634135160914973</v>
       </c>
       <c r="K16" t="n">
-        <v>-1.486111312442224</v>
+        <v>-1.486111402212552</v>
       </c>
     </row>
   </sheetData>

</xml_diff>